<commit_message>
Actualizacion pedidos 22.10: datos comerciales, MRP, tesoreria y rentabilidad
</commit_message>
<xml_diff>
--- a/Pedidos21.10 comerciales.xlsx
+++ b/Pedidos21.10 comerciales.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroquimicacodiagro365-my.sharepoint.com/personal/oscar_ocampo_codiagro_com/Documents/Escritorio/Presupuesto 2026/Calsif Comerciales/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{DB7404D2-ECE7-4680-B483-C9ED25CF4224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E067876-43CF-486C-90F4-AA7E9E864CCF}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="8_{DB7404D2-ECE7-4680-B483-C9ED25CF4224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41BCD2A4-73EB-402C-8AC6-0BE0DC1355FB}"/>
   <bookViews>
-    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{98158736-BF56-4FFC-90E7-0D5AFB7C782B}"/>
+    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{98158736-BF56-4FFC-90E7-0D5AFB7C782B}"/>
   </bookViews>
   <sheets>
     <sheet name="LineasPedidoCliente" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="DatosExternos_1" localSheetId="0" hidden="1">LineasPedidoCliente!$A$1:$P$112</definedName>
+    <definedName name="DatosExternos_1" localSheetId="0" hidden="1">LineasPedidoCliente!$A$1:$P$133</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="222">
   <si>
     <t>FechaPedido</t>
   </si>
@@ -617,6 +617,105 @@
   </si>
   <si>
     <t>FITOKONTROL CA FLOW, 5 KG</t>
+  </si>
+  <si>
+    <t>430000054</t>
+  </si>
+  <si>
+    <t>JUAN JIMENEZ, SRL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGXK0001     </t>
+  </si>
+  <si>
+    <t>BEY0001</t>
+  </si>
+  <si>
+    <t>BIO0001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B0001        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">C-L0001      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">C-CU0001     </t>
+  </si>
+  <si>
+    <t>A-50(2)0001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-A0005      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-A0001      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">LP0005       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">LP0001       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT0005       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT0001       </t>
+  </si>
+  <si>
+    <t>START20001</t>
+  </si>
+  <si>
+    <t>SS0001</t>
+  </si>
+  <si>
+    <t>FLOR0001</t>
+  </si>
+  <si>
+    <t>AGROXILATO-K, 1 L</t>
+  </si>
+  <si>
+    <t>BERRY-FLOR, 1 L</t>
+  </si>
+  <si>
+    <t>BIORAD-20, 1L</t>
+  </si>
+  <si>
+    <t>BOROCAL,1 L</t>
+  </si>
+  <si>
+    <t>CODIBOR-L, 1 L</t>
+  </si>
+  <si>
+    <t>CODICOBRE, 1 L</t>
+  </si>
+  <si>
+    <t>CODIORGAN-A50, 1 KG</t>
+  </si>
+  <si>
+    <t>FITOLIN-AGRO, 5 L</t>
+  </si>
+  <si>
+    <t>FITOLIN-AGRO, 1 L</t>
+  </si>
+  <si>
+    <t>LAVAPLANT, 5 L</t>
+  </si>
+  <si>
+    <t>LAVAPLANT, 1 L</t>
+  </si>
+  <si>
+    <t>RADISOL STARTER, 1 L</t>
+  </si>
+  <si>
+    <t>SALWAX-CA, 1 KG</t>
+  </si>
+  <si>
+    <t>SPRINTENE CON BORO, 1 L</t>
+  </si>
+  <si>
+    <t>FLORAMEC, 1 LTR.</t>
   </si>
 </sst>
 </file>
@@ -652,12 +751,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -695,6 +792,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="DatosExternos_1" connectionId="1" xr16:uid="{141BEB63-F55C-4AB6-A386-A276D3F7899E}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh nextId="17">
@@ -721,8 +822,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{84A60ACA-9758-4E2F-8714-43288D8F7891}" name="LineasPedidoCliente" displayName="LineasPedidoCliente" ref="A1:P112" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:P112" xr:uid="{6292CA43-A9C0-4280-B40A-9DD133760E8A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{84A60ACA-9758-4E2F-8714-43288D8F7891}" name="LineasPedidoCliente" displayName="LineasPedidoCliente" ref="A1:P133" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:P133" xr:uid="{6292CA43-A9C0-4280-B40A-9DD133760E8A}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P92">
     <sortCondition ref="A1:A92"/>
   </sortState>
@@ -1065,7 +1166,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABDBF8C7-4EF9-4D9B-A009-B6059F02B37C}">
-  <dimension ref="A1:P112"/>
+  <dimension ref="A1:P133"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -6223,20 +6324,19 @@
       <c r="B104">
         <v>2026</v>
       </c>
-      <c r="C104" s="2"/>
       <c r="D104">
         <v>888</v>
       </c>
-      <c r="E104" s="3" t="s">
+      <c r="E104" t="s">
         <v>39</v>
       </c>
-      <c r="F104" s="3" t="s">
+      <c r="F104" t="s">
         <v>40</v>
       </c>
-      <c r="G104" s="4" t="s">
+      <c r="G104" t="s">
         <v>105</v>
       </c>
-      <c r="H104" s="2" t="s">
+      <c r="H104" t="s">
         <v>106</v>
       </c>
       <c r="I104">
@@ -6272,20 +6372,19 @@
       <c r="B105">
         <v>2026</v>
       </c>
-      <c r="C105" s="2"/>
       <c r="D105">
         <v>888</v>
       </c>
-      <c r="E105" s="4" t="s">
+      <c r="E105" t="s">
         <v>39</v>
       </c>
-      <c r="F105" s="4" t="s">
+      <c r="F105" t="s">
         <v>40</v>
       </c>
-      <c r="G105" s="4" t="s">
+      <c r="G105" t="s">
         <v>103</v>
       </c>
-      <c r="H105" s="2" t="s">
+      <c r="H105" t="s">
         <v>104</v>
       </c>
       <c r="I105">
@@ -6303,7 +6402,7 @@
       <c r="M105">
         <v>0</v>
       </c>
-      <c r="N105" s="4">
+      <c r="N105">
         <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
         <v>2002</v>
       </c>
@@ -6321,20 +6420,19 @@
       <c r="B106">
         <v>2026</v>
       </c>
-      <c r="C106" s="2"/>
       <c r="D106">
         <v>888</v>
       </c>
-      <c r="E106" s="4" t="s">
+      <c r="E106" t="s">
         <v>39</v>
       </c>
-      <c r="F106" s="4" t="s">
+      <c r="F106" t="s">
         <v>40</v>
       </c>
-      <c r="G106" s="4" t="s">
+      <c r="G106" t="s">
         <v>41</v>
       </c>
-      <c r="H106" s="2" t="s">
+      <c r="H106" t="s">
         <v>42</v>
       </c>
       <c r="I106">
@@ -6352,7 +6450,7 @@
       <c r="M106">
         <v>0</v>
       </c>
-      <c r="N106" s="4">
+      <c r="N106">
         <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
         <v>803.99999999999989</v>
       </c>
@@ -6370,20 +6468,19 @@
       <c r="B107">
         <v>2026</v>
       </c>
-      <c r="C107" s="2"/>
       <c r="D107">
         <v>888</v>
       </c>
-      <c r="E107" s="4" t="s">
+      <c r="E107" t="s">
         <v>39</v>
       </c>
-      <c r="F107" s="4" t="s">
+      <c r="F107" t="s">
         <v>40</v>
       </c>
-      <c r="G107" s="4" t="s">
+      <c r="G107" t="s">
         <v>47</v>
       </c>
-      <c r="H107" s="2" t="s">
+      <c r="H107" t="s">
         <v>48</v>
       </c>
       <c r="I107">
@@ -6401,7 +6498,7 @@
       <c r="M107">
         <v>0</v>
       </c>
-      <c r="N107" s="4">
+      <c r="N107">
         <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
         <v>1344</v>
       </c>
@@ -6419,20 +6516,19 @@
       <c r="B108">
         <v>2026</v>
       </c>
-      <c r="C108" s="2"/>
       <c r="D108">
         <v>888</v>
       </c>
-      <c r="E108" s="4" t="s">
+      <c r="E108" t="s">
         <v>39</v>
       </c>
-      <c r="F108" s="4" t="s">
+      <c r="F108" t="s">
         <v>40</v>
       </c>
-      <c r="G108" s="4" t="s">
+      <c r="G108" t="s">
         <v>41</v>
       </c>
-      <c r="H108" s="2" t="s">
+      <c r="H108" t="s">
         <v>42</v>
       </c>
       <c r="I108">
@@ -6450,7 +6546,7 @@
       <c r="M108">
         <v>0</v>
       </c>
-      <c r="N108" s="4">
+      <c r="N108">
         <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
         <v>4019.9999999999995</v>
       </c>
@@ -6465,23 +6561,22 @@
       <c r="A109" s="1">
         <v>46315</v>
       </c>
-      <c r="B109" s="4">
-        <v>2026</v>
-      </c>
-      <c r="C109" s="2"/>
+      <c r="B109">
+        <v>2026</v>
+      </c>
       <c r="D109">
         <v>889</v>
       </c>
-      <c r="E109" s="2">
+      <c r="E109">
         <v>430000429</v>
       </c>
-      <c r="F109" s="2" t="s">
+      <c r="F109" t="s">
         <v>84</v>
       </c>
-      <c r="G109" s="2" t="s">
+      <c r="G109" t="s">
         <v>187</v>
       </c>
-      <c r="H109" s="2" t="s">
+      <c r="H109" t="s">
         <v>188</v>
       </c>
       <c r="I109">
@@ -6514,23 +6609,22 @@
       <c r="A110" s="1">
         <v>46315</v>
       </c>
-      <c r="B110" s="4">
-        <v>2026</v>
-      </c>
-      <c r="C110" s="2"/>
-      <c r="D110" s="4">
+      <c r="B110">
+        <v>2026</v>
+      </c>
+      <c r="D110">
         <v>889</v>
       </c>
-      <c r="E110" s="2">
+      <c r="E110">
         <v>430000429</v>
       </c>
-      <c r="F110" s="2" t="s">
+      <c r="F110" t="s">
         <v>84</v>
       </c>
-      <c r="G110" s="2" t="s">
+      <c r="G110" t="s">
         <v>151</v>
       </c>
-      <c r="H110" s="2" t="s">
+      <c r="H110" t="s">
         <v>152</v>
       </c>
       <c r="I110">
@@ -6548,7 +6642,7 @@
       <c r="M110">
         <v>0</v>
       </c>
-      <c r="N110" s="5">
+      <c r="N110">
         <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
         <v>222.00000000000003</v>
       </c>
@@ -6563,23 +6657,22 @@
       <c r="A111" s="1">
         <v>46315</v>
       </c>
-      <c r="B111" s="4">
-        <v>2026</v>
-      </c>
-      <c r="C111" s="2"/>
-      <c r="D111" s="4">
+      <c r="B111">
+        <v>2026</v>
+      </c>
+      <c r="D111">
         <v>889</v>
       </c>
-      <c r="E111" s="2">
+      <c r="E111">
         <v>430000429</v>
       </c>
-      <c r="F111" s="2" t="s">
+      <c r="F111" t="s">
         <v>84</v>
       </c>
-      <c r="G111" s="2" t="s">
+      <c r="G111" t="s">
         <v>73</v>
       </c>
-      <c r="H111" s="2" t="s">
+      <c r="H111" t="s">
         <v>74</v>
       </c>
       <c r="I111">
@@ -6597,7 +6690,7 @@
       <c r="M111">
         <v>0</v>
       </c>
-      <c r="N111" s="5">
+      <c r="N111">
         <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
         <v>316</v>
       </c>
@@ -6612,23 +6705,22 @@
       <c r="A112" s="1">
         <v>46315</v>
       </c>
-      <c r="B112" s="4">
-        <v>2026</v>
-      </c>
-      <c r="C112" s="2"/>
-      <c r="D112" s="4">
+      <c r="B112">
+        <v>2026</v>
+      </c>
+      <c r="D112">
         <v>889</v>
       </c>
-      <c r="E112" s="2">
+      <c r="E112">
         <v>430000429</v>
       </c>
-      <c r="F112" s="2" t="s">
+      <c r="F112" t="s">
         <v>84</v>
       </c>
-      <c r="G112" s="2" t="s">
+      <c r="G112" t="s">
         <v>95</v>
       </c>
-      <c r="H112" s="2" t="s">
+      <c r="H112" t="s">
         <v>96</v>
       </c>
       <c r="I112">
@@ -6646,7 +6738,7 @@
       <c r="M112">
         <v>0</v>
       </c>
-      <c r="N112" s="5">
+      <c r="N112">
         <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
         <v>468</v>
       </c>
@@ -6655,6 +6747,930 @@
       </c>
       <c r="P112">
         <v>2</v>
+      </c>
+    </row>
+    <row r="113" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A113" s="1"/>
+      <c r="C113" s="2"/>
+      <c r="D113">
+        <v>148</v>
+      </c>
+      <c r="E113" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F113" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G113" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H113" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I113">
+        <v>1800</v>
+      </c>
+      <c r="J113">
+        <v>0</v>
+      </c>
+      <c r="K113">
+        <v>1800</v>
+      </c>
+      <c r="L113">
+        <v>1.88</v>
+      </c>
+      <c r="M113" s="3">
+        <v>0</v>
+      </c>
+      <c r="N113" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>3384</v>
+      </c>
+      <c r="O113">
+        <v>3384</v>
+      </c>
+      <c r="P113" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A114" s="1"/>
+      <c r="C114" s="2"/>
+      <c r="D114">
+        <v>148</v>
+      </c>
+      <c r="E114" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F114" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G114" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="H114" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="I114">
+        <v>1788</v>
+      </c>
+      <c r="J114">
+        <v>0</v>
+      </c>
+      <c r="K114">
+        <v>1788</v>
+      </c>
+      <c r="L114">
+        <v>3.99</v>
+      </c>
+      <c r="M114" s="3">
+        <v>0</v>
+      </c>
+      <c r="N114" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>7134.1200000000008</v>
+      </c>
+      <c r="O114">
+        <v>7134.1200000000008</v>
+      </c>
+      <c r="P114" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A115" s="1"/>
+      <c r="C115" s="2"/>
+      <c r="D115">
+        <v>148</v>
+      </c>
+      <c r="E115" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F115" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G115" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="H115" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="I115">
+        <v>36</v>
+      </c>
+      <c r="J115">
+        <v>0</v>
+      </c>
+      <c r="K115">
+        <v>36</v>
+      </c>
+      <c r="L115">
+        <v>4.74</v>
+      </c>
+      <c r="M115" s="3">
+        <v>0</v>
+      </c>
+      <c r="N115" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>170.64000000000001</v>
+      </c>
+      <c r="O115">
+        <v>170.64000000000001</v>
+      </c>
+      <c r="P115" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A116" s="1"/>
+      <c r="C116" s="2"/>
+      <c r="D116">
+        <v>148</v>
+      </c>
+      <c r="E116" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F116" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G116" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="H116" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="I116">
+        <v>3900</v>
+      </c>
+      <c r="J116">
+        <v>0</v>
+      </c>
+      <c r="K116">
+        <v>3900</v>
+      </c>
+      <c r="L116">
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="M116" s="3">
+        <v>0</v>
+      </c>
+      <c r="N116" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>9633</v>
+      </c>
+      <c r="O116">
+        <v>9633</v>
+      </c>
+      <c r="P116" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A117" s="1"/>
+      <c r="C117" s="2"/>
+      <c r="D117">
+        <v>148</v>
+      </c>
+      <c r="E117" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F117" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G117" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H117" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="I117">
+        <v>6400</v>
+      </c>
+      <c r="J117">
+        <v>0</v>
+      </c>
+      <c r="K117">
+        <v>6400</v>
+      </c>
+      <c r="L117">
+        <v>2.39</v>
+      </c>
+      <c r="M117" s="3">
+        <v>0</v>
+      </c>
+      <c r="N117" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>15296</v>
+      </c>
+      <c r="O117">
+        <v>15296</v>
+      </c>
+      <c r="P117" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A118" s="1"/>
+      <c r="C118" s="2"/>
+      <c r="D118">
+        <v>148</v>
+      </c>
+      <c r="E118" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F118" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G118" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="H118" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="I118">
+        <v>2892</v>
+      </c>
+      <c r="J118">
+        <v>0</v>
+      </c>
+      <c r="K118">
+        <v>2892</v>
+      </c>
+      <c r="L118">
+        <v>3.5</v>
+      </c>
+      <c r="M118" s="3">
+        <v>0</v>
+      </c>
+      <c r="N118" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>10122</v>
+      </c>
+      <c r="O118">
+        <v>10122</v>
+      </c>
+      <c r="P118" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A119" s="1"/>
+      <c r="C119" s="2"/>
+      <c r="D119">
+        <v>148</v>
+      </c>
+      <c r="E119" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F119" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G119" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="H119" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="I119">
+        <v>2808</v>
+      </c>
+      <c r="J119">
+        <v>0</v>
+      </c>
+      <c r="K119">
+        <v>2808</v>
+      </c>
+      <c r="L119">
+        <v>4.75</v>
+      </c>
+      <c r="M119" s="3">
+        <v>0</v>
+      </c>
+      <c r="N119" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>13338</v>
+      </c>
+      <c r="O119">
+        <v>13338</v>
+      </c>
+      <c r="P119" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A120" s="1"/>
+      <c r="C120" s="2"/>
+      <c r="D120">
+        <v>148</v>
+      </c>
+      <c r="E120" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F120" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G120" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="H120" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="I120">
+        <v>480</v>
+      </c>
+      <c r="J120">
+        <v>0</v>
+      </c>
+      <c r="K120">
+        <v>480</v>
+      </c>
+      <c r="L120">
+        <v>2.42</v>
+      </c>
+      <c r="M120" s="3">
+        <v>0</v>
+      </c>
+      <c r="N120" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>1161.5999999999999</v>
+      </c>
+      <c r="O120">
+        <v>1161.5999999999999</v>
+      </c>
+      <c r="P120" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A121" s="1"/>
+      <c r="C121" s="2"/>
+      <c r="D121">
+        <v>148</v>
+      </c>
+      <c r="E121" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F121" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G121" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="H121" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="I121">
+        <v>84</v>
+      </c>
+      <c r="J121">
+        <v>0</v>
+      </c>
+      <c r="K121">
+        <v>84</v>
+      </c>
+      <c r="L121">
+        <v>5.58</v>
+      </c>
+      <c r="M121" s="3">
+        <v>0</v>
+      </c>
+      <c r="N121" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>468.72</v>
+      </c>
+      <c r="O121">
+        <v>468.72</v>
+      </c>
+      <c r="P121" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A122" s="1"/>
+      <c r="C122" s="2"/>
+      <c r="D122">
+        <v>148</v>
+      </c>
+      <c r="E122" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F122" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G122" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="H122" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="I122">
+        <v>1200</v>
+      </c>
+      <c r="J122">
+        <v>0</v>
+      </c>
+      <c r="K122">
+        <v>1200</v>
+      </c>
+      <c r="L122">
+        <v>4.83</v>
+      </c>
+      <c r="M122" s="3">
+        <v>0</v>
+      </c>
+      <c r="N122" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>5796</v>
+      </c>
+      <c r="O122">
+        <v>5796</v>
+      </c>
+      <c r="P122" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A123" s="1"/>
+      <c r="C123" s="2"/>
+      <c r="D123">
+        <v>148</v>
+      </c>
+      <c r="E123" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F123" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G123" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="H123" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="I123">
+        <v>2448</v>
+      </c>
+      <c r="J123">
+        <v>0</v>
+      </c>
+      <c r="K123">
+        <v>2448</v>
+      </c>
+      <c r="L123">
+        <v>5.31</v>
+      </c>
+      <c r="M123" s="3">
+        <v>0</v>
+      </c>
+      <c r="N123" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>12998.88</v>
+      </c>
+      <c r="O123">
+        <v>12998.88</v>
+      </c>
+      <c r="P123" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A124" s="1"/>
+      <c r="C124" s="2"/>
+      <c r="D124">
+        <v>148</v>
+      </c>
+      <c r="E124" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F124" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G124" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="H124" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="I124">
+        <v>2040</v>
+      </c>
+      <c r="J124">
+        <v>0</v>
+      </c>
+      <c r="K124">
+        <v>2040</v>
+      </c>
+      <c r="L124">
+        <v>4.7699999999999996</v>
+      </c>
+      <c r="M124" s="3">
+        <v>0</v>
+      </c>
+      <c r="N124" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>9730.7999999999993</v>
+      </c>
+      <c r="O124">
+        <v>9730.7999999999993</v>
+      </c>
+      <c r="P124" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A125" s="1"/>
+      <c r="C125" s="2"/>
+      <c r="D125">
+        <v>148</v>
+      </c>
+      <c r="E125" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F125" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G125" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="H125" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="I125">
+        <v>984</v>
+      </c>
+      <c r="J125">
+        <v>0</v>
+      </c>
+      <c r="K125">
+        <v>984</v>
+      </c>
+      <c r="L125">
+        <v>5.78</v>
+      </c>
+      <c r="M125" s="3">
+        <v>0</v>
+      </c>
+      <c r="N125" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>5687.52</v>
+      </c>
+      <c r="O125">
+        <v>5687.52</v>
+      </c>
+      <c r="P125" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A126" s="1"/>
+      <c r="C126" s="2"/>
+      <c r="D126">
+        <v>148</v>
+      </c>
+      <c r="E126" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F126" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G126" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="H126" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="I126">
+        <v>1160</v>
+      </c>
+      <c r="J126">
+        <v>0</v>
+      </c>
+      <c r="K126">
+        <v>1160</v>
+      </c>
+      <c r="L126">
+        <v>3.74</v>
+      </c>
+      <c r="M126" s="3">
+        <v>0</v>
+      </c>
+      <c r="N126" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>4338.4000000000005</v>
+      </c>
+      <c r="O126">
+        <v>4338.4000000000005</v>
+      </c>
+      <c r="P126" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A127" s="1"/>
+      <c r="C127" s="2"/>
+      <c r="D127">
+        <v>148</v>
+      </c>
+      <c r="E127" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F127" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G127" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="H127" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="I127">
+        <v>1092</v>
+      </c>
+      <c r="J127">
+        <v>0</v>
+      </c>
+      <c r="K127">
+        <v>1092</v>
+      </c>
+      <c r="L127">
+        <v>4.68</v>
+      </c>
+      <c r="M127" s="3">
+        <v>0</v>
+      </c>
+      <c r="N127" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>5110.5599999999995</v>
+      </c>
+      <c r="O127">
+        <v>5110.5599999999995</v>
+      </c>
+      <c r="P127" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A128" s="1"/>
+      <c r="C128" s="2"/>
+      <c r="D128">
+        <v>148</v>
+      </c>
+      <c r="E128" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F128" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G128" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="H128" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="I128">
+        <v>1260</v>
+      </c>
+      <c r="J128">
+        <v>0</v>
+      </c>
+      <c r="K128">
+        <v>1260</v>
+      </c>
+      <c r="L128">
+        <v>3.21</v>
+      </c>
+      <c r="M128" s="3">
+        <v>0</v>
+      </c>
+      <c r="N128" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>4044.6</v>
+      </c>
+      <c r="O128">
+        <v>4044.6</v>
+      </c>
+      <c r="P128" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A129" s="1"/>
+      <c r="C129" s="2"/>
+      <c r="D129">
+        <v>148</v>
+      </c>
+      <c r="E129" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F129" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G129" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="H129" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="I129">
+        <v>2520</v>
+      </c>
+      <c r="J129">
+        <v>0</v>
+      </c>
+      <c r="K129">
+        <v>2520</v>
+      </c>
+      <c r="L129">
+        <v>4.16</v>
+      </c>
+      <c r="M129" s="3">
+        <v>0</v>
+      </c>
+      <c r="N129" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>10483.200000000001</v>
+      </c>
+      <c r="O129">
+        <v>10483.200000000001</v>
+      </c>
+      <c r="P129" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A130" s="1"/>
+      <c r="C130" s="2"/>
+      <c r="D130">
+        <v>148</v>
+      </c>
+      <c r="E130" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F130" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G130" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="H130" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="I130">
+        <v>2904</v>
+      </c>
+      <c r="J130">
+        <v>0</v>
+      </c>
+      <c r="K130">
+        <v>2904</v>
+      </c>
+      <c r="L130">
+        <v>5.87</v>
+      </c>
+      <c r="M130" s="3">
+        <v>0</v>
+      </c>
+      <c r="N130" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>17046.48</v>
+      </c>
+      <c r="O130">
+        <v>17046.48</v>
+      </c>
+      <c r="P130" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A131" s="1"/>
+      <c r="C131" s="2"/>
+      <c r="D131">
+        <v>148</v>
+      </c>
+      <c r="E131" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F131" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G131" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="H131" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="I131">
+        <v>1088</v>
+      </c>
+      <c r="J131">
+        <v>0</v>
+      </c>
+      <c r="K131">
+        <v>1088</v>
+      </c>
+      <c r="L131">
+        <v>4.53</v>
+      </c>
+      <c r="M131" s="3">
+        <v>0</v>
+      </c>
+      <c r="N131" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>4928.6400000000003</v>
+      </c>
+      <c r="O131">
+        <v>4928.6400000000003</v>
+      </c>
+      <c r="P131" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A132" s="1"/>
+      <c r="C132" s="2"/>
+      <c r="D132">
+        <v>148</v>
+      </c>
+      <c r="E132" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F132" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G132" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="H132" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="I132">
+        <v>300</v>
+      </c>
+      <c r="J132">
+        <v>0</v>
+      </c>
+      <c r="K132">
+        <v>300</v>
+      </c>
+      <c r="L132">
+        <v>12.83</v>
+      </c>
+      <c r="M132" s="3">
+        <v>0</v>
+      </c>
+      <c r="N132" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>3849</v>
+      </c>
+      <c r="O132">
+        <v>3849</v>
+      </c>
+      <c r="P132" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A133" s="1"/>
+      <c r="C133" s="2"/>
+      <c r="D133">
+        <v>148</v>
+      </c>
+      <c r="E133" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="F133" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="G133" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="H133" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="I133">
+        <v>648</v>
+      </c>
+      <c r="J133">
+        <v>0</v>
+      </c>
+      <c r="K133">
+        <v>648</v>
+      </c>
+      <c r="L133">
+        <v>3.83</v>
+      </c>
+      <c r="M133" s="3">
+        <v>0</v>
+      </c>
+      <c r="N133" s="3">
+        <f>LineasPedidoCliente[[#This Row],[Pedidas]]*LineasPedidoCliente[[#This Row],[Precio]]</f>
+        <v>2481.84</v>
+      </c>
+      <c r="O133">
+        <v>2481.84</v>
+      </c>
+      <c r="P133" s="3">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>